<commit_message>
Added new student list in this .xlsx file
</commit_message>
<xml_diff>
--- a/students.xlsx
+++ b/students.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HarnPhomn\Desktop\Git Clone\git-intro-lms\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e9e534bb53071102/Desktop/Git Clone/git-intro-lms/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FADFB1A5-3936-412C-92BC-ED70A2187C9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{FADFB1A5-3936-412C-92BC-ED70A2187C9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9DC08486-3463-4044-96CE-A993E04A394B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
   <si>
     <t>ၸိုဝ်ႈ</t>
   </si>
@@ -61,6 +61,15 @@
   </si>
   <si>
     <t>han845457@gmail.com</t>
+  </si>
+  <si>
+    <t>ၸဝ်ႈသၢင်ႇ မႃႇၼိတ</t>
+  </si>
+  <si>
+    <t>မိူင်းႁႃႉ</t>
+  </si>
+  <si>
+    <t>artificialmgphone@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -137,9 +146,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -177,7 +186,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -283,7 +292,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -425,7 +434,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -433,8 +442,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.2"/>
+  <cols>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
@@ -476,12 +488,27 @@
       </c>
       <c r="D3" s="3" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="D3" r:id="rId2" xr:uid="{A2393D93-9977-4865-B646-4C1E1A205BAD}"/>
+    <hyperlink ref="D4" r:id="rId3" xr:uid="{E49C088E-D1FA-4DB9-85EA-1F346E3E91B9}"/>
   </hyperlinks>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>